<commit_message>
removed  home path updated data and added python script
</commit_message>
<xml_diff>
--- a/data/Mu&OffsetData.xlsx
+++ b/data/Mu&OffsetData.xlsx
@@ -205,13 +205,13 @@
     <t>0.69359566,</t>
   </si>
   <si>
-    <t>Cardboard MAE: 0.12204189921964285</t>
+    <t>Cardboard MAE: 0.12099004850535715</t>
   </si>
   <si>
     <t>0.66521889,</t>
   </si>
   <si>
-    <t>Cardboard MRE %: 11.964892080357144</t>
+    <t>Cardboard MRE %: 11.746606651005546</t>
   </si>
   <si>
     <t>0.6785552684,</t>
@@ -700,7 +700,7 @@
     <t>true_tile_mu = 0.69</t>
   </si>
   <si>
-    <t>true_cardboard_mu = 1.02</t>
+    <t>true_cardboard_mu = 1.03</t>
   </si>
   <si>
     <t>true_acrylic_mu = 0.84</t>
@@ -1290,7 +1290,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1329,6 +1329,9 @@
     </xf>
     <xf borderId="12" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="12" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="13" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
@@ -4346,7 +4349,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="20" t="s">
         <v>54</v>
       </c>
       <c r="I2" s="1" t="s">
@@ -4354,7 +4357,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="20" t="s">
         <v>56</v>
       </c>
       <c r="I3" s="1" t="s">
@@ -4362,7 +4365,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="20" t="s">
         <v>58</v>
       </c>
       <c r="I4" s="1" t="s">
@@ -4370,7 +4373,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="20" t="s">
         <v>60</v>
       </c>
       <c r="I5" s="1" t="s">
@@ -4378,7 +4381,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="20" t="s">
         <v>62</v>
       </c>
       <c r="I6" s="1" t="s">
@@ -4386,7 +4389,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="20" t="s">
         <v>64</v>
       </c>
       <c r="I7" s="1" t="s">
@@ -4397,7 +4400,7 @@
       <c r="A8" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="20" t="s">
         <v>67</v>
       </c>
       <c r="I8" s="1" t="s">
@@ -4408,7 +4411,7 @@
       <c r="A9" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="20" t="s">
         <v>70</v>
       </c>
       <c r="I9" s="1" t="s">
@@ -4416,7 +4419,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="20" t="s">
         <v>72</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -5413,10 +5416,10 @@
       <c r="K4" s="1">
         <v>0.990763230536271</v>
       </c>
-      <c r="N4" s="20" t="s">
+      <c r="N4" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="21"/>
+      <c r="O4" s="22"/>
     </row>
     <row r="5">
       <c r="F5" s="1" t="s">
@@ -6486,14 +6489,14 @@
       <c r="G44" s="1">
         <v>12.898</v>
       </c>
-      <c r="H44" s="22">
+      <c r="H44" s="23">
         <v>1.77076115752053E9</v>
       </c>
       <c r="I44" s="4">
         <f t="shared" si="15"/>
         <v>0.2152712364</v>
       </c>
-      <c r="J44" s="22">
+      <c r="J44" s="23">
         <v>1.0378559732</v>
       </c>
       <c r="K44" s="1">
@@ -6718,7 +6721,7 @@
         <v>11</v>
       </c>
       <c r="K2" s="2"/>
-      <c r="L2" s="23"/>
+      <c r="L2" s="24"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
@@ -6744,7 +6747,7 @@
       <c r="J4" s="1">
         <v>0.7938452464</v>
       </c>
-      <c r="N4" s="24"/>
+      <c r="N4" s="25"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
@@ -6878,7 +6881,7 @@
       <c r="J14" s="1">
         <v>1.0746031465</v>
       </c>
-      <c r="N14" s="24"/>
+      <c r="N14" s="25"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
@@ -6893,9 +6896,9 @@
       <c r="J15" s="1">
         <v>0.7674276654</v>
       </c>
-      <c r="N15" s="24"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="24"/>
+      <c r="N15" s="25"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="25"/>
     </row>
     <row r="16">
       <c r="F16" s="1" t="s">
@@ -7238,15 +7241,15 @@
     </row>
     <row r="52">
       <c r="M52" s="2"/>
-      <c r="N52" s="25"/>
-      <c r="O52" s="25"/>
-      <c r="P52" s="25"/>
+      <c r="N52" s="26"/>
+      <c r="O52" s="26"/>
+      <c r="P52" s="26"/>
     </row>
     <row r="53">
       <c r="M53" s="2"/>
-      <c r="N53" s="25"/>
-      <c r="O53" s="25"/>
-      <c r="P53" s="25"/>
+      <c r="N53" s="26"/>
+      <c r="O53" s="26"/>
+      <c r="P53" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -7303,7 +7306,7 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>274</v>
       </c>
       <c r="L2" s="2"/>
@@ -7324,8 +7327,8 @@
       <c r="E3" s="1">
         <v>0.8415899703</v>
       </c>
-      <c r="J3" s="27"/>
-      <c r="K3" s="28"/>
+      <c r="J3" s="28"/>
+      <c r="K3" s="29"/>
       <c r="M3" s="1" t="s">
         <v>275</v>
       </c>
@@ -7355,8 +7358,8 @@
       <c r="E4" s="1">
         <v>0.9127304548</v>
       </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="28"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="29"/>
       <c r="M4" s="1" t="s">
         <v>281</v>
       </c>
@@ -7386,8 +7389,8 @@
       <c r="E5" s="1">
         <v>0.6960932134</v>
       </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="28"/>
+      <c r="J5" s="28"/>
+      <c r="K5" s="29"/>
       <c r="M5" s="1" t="s">
         <v>286</v>
       </c>
@@ -7411,7 +7414,7 @@
       <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="30">
         <v>2.0</v>
       </c>
       <c r="D6" s="1">
@@ -7420,8 +7423,8 @@
       <c r="E6" s="1">
         <v>1.1257118388</v>
       </c>
-      <c r="J6" s="27"/>
-      <c r="K6" s="28"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="29"/>
       <c r="M6" s="1" t="s">
         <v>291</v>
       </c>
@@ -7451,8 +7454,8 @@
       <c r="E7" s="1">
         <v>0.9801569032</v>
       </c>
-      <c r="J7" s="27"/>
-      <c r="K7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="29"/>
       <c r="M7" s="1" t="s">
         <v>296</v>
       </c>
@@ -7482,8 +7485,8 @@
       <c r="E8" s="1">
         <v>0.711716796</v>
       </c>
-      <c r="J8" s="27"/>
-      <c r="K8" s="28"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="29"/>
       <c r="M8" s="1" t="s">
         <v>301</v>
       </c>
@@ -7516,8 +7519,8 @@
       <c r="E9" s="1">
         <v>1.1714725596</v>
       </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="28"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="29"/>
       <c r="M9" s="1" t="s">
         <v>306</v>
       </c>
@@ -7547,8 +7550,8 @@
       <c r="E10" s="1">
         <v>0.8675244117</v>
       </c>
-      <c r="J10" s="27"/>
-      <c r="K10" s="28"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="29"/>
       <c r="M10" s="1" t="s">
         <v>310</v>
       </c>
@@ -7578,8 +7581,8 @@
       <c r="E11" s="1">
         <v>0.7205852602</v>
       </c>
-      <c r="J11" s="27"/>
-      <c r="K11" s="28"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="29"/>
       <c r="M11" s="1" t="s">
         <v>315</v>
       </c>
@@ -7615,8 +7618,8 @@
       <c r="F12" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="J12" s="27"/>
-      <c r="K12" s="28"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="29"/>
       <c r="M12" s="1" t="s">
         <v>320</v>
       </c>
@@ -7646,8 +7649,8 @@
       <c r="E13" s="1">
         <v>1.0748973615</v>
       </c>
-      <c r="J13" s="27"/>
-      <c r="K13" s="28"/>
+      <c r="J13" s="28"/>
+      <c r="K13" s="29"/>
       <c r="M13" s="1" t="s">
         <v>325</v>
       </c>
@@ -7677,8 +7680,8 @@
       <c r="E14" s="1">
         <v>0.7014588838</v>
       </c>
-      <c r="J14" s="27"/>
-      <c r="K14" s="28"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="29"/>
       <c r="M14" s="1" t="s">
         <v>330</v>
       </c>
@@ -7711,8 +7714,8 @@
       <c r="E15" s="1">
         <v>1.0939337648</v>
       </c>
-      <c r="J15" s="27"/>
-      <c r="K15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="29"/>
       <c r="M15" s="1" t="s">
         <v>334</v>
       </c>
@@ -7742,8 +7745,8 @@
       <c r="E16" s="1">
         <v>0.9176910204</v>
       </c>
-      <c r="J16" s="27"/>
-      <c r="K16" s="28"/>
+      <c r="J16" s="28"/>
+      <c r="K16" s="29"/>
     </row>
     <row r="17">
       <c r="B17" s="1" t="s">
@@ -7758,8 +7761,8 @@
       <c r="E17" s="1">
         <v>0.7630843658</v>
       </c>
-      <c r="J17" s="27"/>
-      <c r="K17" s="28"/>
+      <c r="J17" s="28"/>
+      <c r="K17" s="29"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
@@ -7777,8 +7780,8 @@
       <c r="E18" s="1">
         <v>1.2232984343</v>
       </c>
-      <c r="J18" s="27"/>
-      <c r="K18" s="28"/>
+      <c r="J18" s="28"/>
+      <c r="K18" s="29"/>
     </row>
     <row r="19">
       <c r="B19" s="1" t="s">
@@ -7793,8 +7796,8 @@
       <c r="E19" s="1">
         <v>0.7205485175</v>
       </c>
-      <c r="J19" s="27"/>
-      <c r="K19" s="28"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="29"/>
     </row>
     <row r="20">
       <c r="B20" s="1" t="s">
@@ -7809,8 +7812,8 @@
       <c r="E20" s="1">
         <v>0.65954879</v>
       </c>
-      <c r="J20" s="27"/>
-      <c r="K20" s="28"/>
+      <c r="J20" s="28"/>
+      <c r="K20" s="29"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
@@ -7828,8 +7831,8 @@
       <c r="E21" s="1">
         <v>1.2385643507</v>
       </c>
-      <c r="J21" s="27"/>
-      <c r="K21" s="28"/>
+      <c r="J21" s="28"/>
+      <c r="K21" s="29"/>
     </row>
     <row r="22">
       <c r="B22" s="1" t="s">
@@ -7844,14 +7847,14 @@
       <c r="E22" s="1">
         <v>0.9599639196</v>
       </c>
-      <c r="J22" s="27"/>
-      <c r="K22" s="28"/>
-      <c r="M22" s="30"/>
-      <c r="N22" s="30"/>
-      <c r="P22" s="30"/>
-      <c r="S22" s="30"/>
-      <c r="V22" s="31"/>
-      <c r="Y22" s="31"/>
+      <c r="J22" s="28"/>
+      <c r="K22" s="29"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="31"/>
+      <c r="P22" s="31"/>
+      <c r="S22" s="31"/>
+      <c r="V22" s="32"/>
+      <c r="Y22" s="32"/>
     </row>
     <row r="23">
       <c r="B23" s="1" t="s">
@@ -7866,12 +7869,12 @@
       <c r="E23" s="1">
         <v>0.6950948899</v>
       </c>
-      <c r="J23" s="27"/>
-      <c r="K23" s="28"/>
-      <c r="V23" s="32"/>
-      <c r="W23" s="32"/>
-      <c r="Y23" s="32"/>
-      <c r="Z23" s="32"/>
+      <c r="J23" s="28"/>
+      <c r="K23" s="29"/>
+      <c r="V23" s="33"/>
+      <c r="W23" s="33"/>
+      <c r="Y23" s="33"/>
+      <c r="Z23" s="33"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
@@ -7889,8 +7892,8 @@
       <c r="E24" s="1">
         <v>1.207087062</v>
       </c>
-      <c r="J24" s="27"/>
-      <c r="K24" s="28"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="29"/>
     </row>
     <row r="25">
       <c r="B25" s="1" t="s">
@@ -7905,8 +7908,8 @@
       <c r="E25" s="1">
         <v>0.9006794133</v>
       </c>
-      <c r="J25" s="27"/>
-      <c r="K25" s="28"/>
+      <c r="J25" s="28"/>
+      <c r="K25" s="29"/>
     </row>
     <row r="26">
       <c r="B26" s="1" t="s">
@@ -7921,8 +7924,8 @@
       <c r="E26" s="1">
         <v>0.6912420848</v>
       </c>
-      <c r="J26" s="27"/>
-      <c r="K26" s="28"/>
+      <c r="J26" s="28"/>
+      <c r="K26" s="29"/>
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
@@ -7940,8 +7943,8 @@
       <c r="E27" s="1">
         <v>1.12737686318637</v>
       </c>
-      <c r="J27" s="27"/>
-      <c r="K27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="29"/>
     </row>
     <row r="28">
       <c r="B28" s="1" t="s">
@@ -7956,8 +7959,8 @@
       <c r="E28" s="1">
         <v>1.10586810208812</v>
       </c>
-      <c r="J28" s="27"/>
-      <c r="K28" s="28"/>
+      <c r="J28" s="28"/>
+      <c r="K28" s="29"/>
     </row>
     <row r="29">
       <c r="B29" s="1" t="s">
@@ -7972,8 +7975,8 @@
       <c r="E29" s="1">
         <v>0.750480501517266</v>
       </c>
-      <c r="J29" s="27"/>
-      <c r="K29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="29"/>
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
@@ -7991,8 +7994,8 @@
       <c r="E30" s="1">
         <v>0.928818455</v>
       </c>
-      <c r="J30" s="27"/>
-      <c r="K30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="29"/>
     </row>
     <row r="31">
       <c r="B31" s="1" t="s">
@@ -8007,8 +8010,8 @@
       <c r="E31" s="1">
         <v>0.6981543221</v>
       </c>
-      <c r="J31" s="27"/>
-      <c r="K31" s="28"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="29"/>
     </row>
     <row r="32">
       <c r="B32" s="1" t="s">
@@ -8023,8 +8026,8 @@
       <c r="E32" s="1">
         <v>0.6795514235</v>
       </c>
-      <c r="J32" s="27"/>
-      <c r="K32" s="28"/>
+      <c r="J32" s="28"/>
+      <c r="K32" s="29"/>
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
@@ -8042,8 +8045,8 @@
       <c r="E33" s="1">
         <v>1.0654395648</v>
       </c>
-      <c r="J33" s="27"/>
-      <c r="K33" s="28"/>
+      <c r="J33" s="28"/>
+      <c r="K33" s="29"/>
     </row>
     <row r="34">
       <c r="B34" s="1" t="s">
@@ -8058,8 +8061,8 @@
       <c r="E34" s="1">
         <v>0.7520148837</v>
       </c>
-      <c r="J34" s="27"/>
-      <c r="K34" s="28"/>
+      <c r="J34" s="28"/>
+      <c r="K34" s="29"/>
     </row>
     <row r="35">
       <c r="B35" s="1" t="s">
@@ -8074,8 +8077,8 @@
       <c r="E35" s="1">
         <v>0.7371280318</v>
       </c>
-      <c r="J35" s="27"/>
-      <c r="K35" s="28"/>
+      <c r="J35" s="28"/>
+      <c r="K35" s="29"/>
     </row>
     <row r="36">
       <c r="A36" s="1" t="s">
@@ -8093,8 +8096,8 @@
       <c r="E36" s="1">
         <v>1.0844269984</v>
       </c>
-      <c r="J36" s="27"/>
-      <c r="K36" s="28"/>
+      <c r="J36" s="28"/>
+      <c r="K36" s="29"/>
     </row>
     <row r="37">
       <c r="B37" s="1" t="s">
@@ -8109,8 +8112,8 @@
       <c r="E37" s="1">
         <v>0.9668405456</v>
       </c>
-      <c r="J37" s="27"/>
-      <c r="K37" s="28"/>
+      <c r="J37" s="28"/>
+      <c r="K37" s="29"/>
     </row>
     <row r="38">
       <c r="B38" s="1" t="s">
@@ -8125,8 +8128,8 @@
       <c r="E38" s="1">
         <v>0.6586842966</v>
       </c>
-      <c r="J38" s="27"/>
-      <c r="K38" s="28"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="29"/>
     </row>
     <row r="39">
       <c r="A39" s="1" t="s">
@@ -8144,8 +8147,8 @@
       <c r="E39" s="1">
         <v>1.0026714958</v>
       </c>
-      <c r="J39" s="27"/>
-      <c r="K39" s="28"/>
+      <c r="J39" s="28"/>
+      <c r="K39" s="29"/>
     </row>
     <row r="40">
       <c r="B40" s="1" t="s">
@@ -8160,8 +8163,8 @@
       <c r="E40" s="1">
         <v>0.7233920819</v>
       </c>
-      <c r="J40" s="27"/>
-      <c r="K40" s="28"/>
+      <c r="J40" s="28"/>
+      <c r="K40" s="29"/>
     </row>
     <row r="41">
       <c r="B41" s="1" t="s">
@@ -8176,8 +8179,8 @@
       <c r="E41" s="1">
         <v>0.7251524385</v>
       </c>
-      <c r="J41" s="27"/>
-      <c r="K41" s="28"/>
+      <c r="J41" s="28"/>
+      <c r="K41" s="29"/>
     </row>
     <row r="42">
       <c r="A42" s="1" t="s">
@@ -8195,8 +8198,8 @@
       <c r="E42" s="1">
         <v>0.9468346919</v>
       </c>
-      <c r="J42" s="27"/>
-      <c r="K42" s="28"/>
+      <c r="J42" s="28"/>
+      <c r="K42" s="29"/>
     </row>
     <row r="43">
       <c r="B43" s="1" t="s">
@@ -8211,8 +8214,8 @@
       <c r="E43" s="1">
         <v>1.0436262687</v>
       </c>
-      <c r="J43" s="27"/>
-      <c r="K43" s="28"/>
+      <c r="J43" s="28"/>
+      <c r="K43" s="29"/>
     </row>
     <row r="44">
       <c r="B44" s="1" t="s">
@@ -8227,8 +8230,8 @@
       <c r="E44" s="1">
         <v>0.6678314216</v>
       </c>
-      <c r="J44" s="27"/>
-      <c r="K44" s="28"/>
+      <c r="J44" s="28"/>
+      <c r="K44" s="29"/>
     </row>
     <row r="45">
       <c r="A45" s="1" t="s">
@@ -8246,8 +8249,8 @@
       <c r="E45" s="1">
         <v>1.0486527015</v>
       </c>
-      <c r="J45" s="27"/>
-      <c r="K45" s="28"/>
+      <c r="J45" s="28"/>
+      <c r="K45" s="29"/>
     </row>
     <row r="46">
       <c r="B46" s="1" t="s">
@@ -8262,8 +8265,8 @@
       <c r="E46" s="1">
         <v>0.7675737622</v>
       </c>
-      <c r="J46" s="27"/>
-      <c r="K46" s="28"/>
+      <c r="J46" s="28"/>
+      <c r="K46" s="29"/>
     </row>
     <row r="47">
       <c r="B47" s="1" t="s">
@@ -8278,8 +8281,8 @@
       <c r="E47" s="1">
         <v>0.6395216272</v>
       </c>
-      <c r="J47" s="27"/>
-      <c r="K47" s="28"/>
+      <c r="J47" s="28"/>
+      <c r="K47" s="29"/>
     </row>
     <row r="48">
       <c r="A48" s="1" t="s">
@@ -8297,8 +8300,8 @@
       <c r="E48" s="1">
         <v>0.9765088555</v>
       </c>
-      <c r="J48" s="27"/>
-      <c r="K48" s="28"/>
+      <c r="J48" s="28"/>
+      <c r="K48" s="29"/>
     </row>
     <row r="49">
       <c r="B49" s="1" t="s">
@@ -8313,8 +8316,8 @@
       <c r="E49" s="1">
         <v>0.6747166092</v>
       </c>
-      <c r="J49" s="27"/>
-      <c r="K49" s="28"/>
+      <c r="J49" s="28"/>
+      <c r="K49" s="29"/>
     </row>
     <row r="50">
       <c r="B50" s="1" t="s">
@@ -8329,8 +8332,8 @@
       <c r="E50" s="1">
         <v>0.630516063</v>
       </c>
-      <c r="J50" s="27"/>
-      <c r="K50" s="28"/>
+      <c r="J50" s="28"/>
+      <c r="K50" s="29"/>
     </row>
     <row r="51">
       <c r="A51" s="1" t="s">
@@ -8351,8 +8354,8 @@
       <c r="F51" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="J51" s="27"/>
-      <c r="K51" s="28"/>
+      <c r="J51" s="28"/>
+      <c r="K51" s="29"/>
     </row>
     <row r="52">
       <c r="B52" s="1" t="s">
@@ -8367,8 +8370,8 @@
       <c r="E52" s="1">
         <v>0.6826693048</v>
       </c>
-      <c r="J52" s="27"/>
-      <c r="K52" s="28"/>
+      <c r="J52" s="28"/>
+      <c r="K52" s="29"/>
     </row>
     <row r="53">
       <c r="B53" s="1" t="s">
@@ -8383,8 +8386,8 @@
       <c r="E53" s="1">
         <v>0.5967960455</v>
       </c>
-      <c r="J53" s="27"/>
-      <c r="K53" s="28"/>
+      <c r="J53" s="28"/>
+      <c r="K53" s="29"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="s">
@@ -8402,8 +8405,8 @@
       <c r="E54" s="1">
         <v>0.9142219725</v>
       </c>
-      <c r="J54" s="27"/>
-      <c r="K54" s="28"/>
+      <c r="J54" s="28"/>
+      <c r="K54" s="29"/>
     </row>
     <row r="55">
       <c r="B55" s="1" t="s">
@@ -8418,8 +8421,8 @@
       <c r="E55" s="1">
         <v>0.722906372</v>
       </c>
-      <c r="J55" s="27"/>
-      <c r="K55" s="28"/>
+      <c r="J55" s="28"/>
+      <c r="K55" s="29"/>
     </row>
     <row r="56">
       <c r="B56" s="1" t="s">
@@ -8434,8 +8437,8 @@
       <c r="E56" s="1">
         <v>0.6952665292</v>
       </c>
-      <c r="J56" s="27"/>
-      <c r="K56" s="28"/>
+      <c r="J56" s="28"/>
+      <c r="K56" s="29"/>
     </row>
     <row r="57">
       <c r="A57" s="1" t="s">
@@ -8453,8 +8456,8 @@
       <c r="E57" s="1">
         <v>0.936962369024282</v>
       </c>
-      <c r="J57" s="27"/>
-      <c r="K57" s="28"/>
+      <c r="J57" s="28"/>
+      <c r="K57" s="29"/>
     </row>
     <row r="58">
       <c r="B58" s="1" t="s">
@@ -8469,8 +8472,8 @@
       <c r="E58" s="1">
         <v>1.06170511115125</v>
       </c>
-      <c r="J58" s="27"/>
-      <c r="K58" s="28"/>
+      <c r="J58" s="28"/>
+      <c r="K58" s="29"/>
     </row>
     <row r="59">
       <c r="B59" s="1" t="s">
@@ -8485,8 +8488,8 @@
       <c r="E59" s="1">
         <v>0.699887318630538</v>
       </c>
-      <c r="J59" s="27"/>
-      <c r="K59" s="28"/>
+      <c r="J59" s="28"/>
+      <c r="K59" s="29"/>
     </row>
     <row r="60">
       <c r="A60" s="1" t="s">
@@ -8504,8 +8507,8 @@
       <c r="E60" s="1">
         <v>1.02945181978471</v>
       </c>
-      <c r="J60" s="27"/>
-      <c r="K60" s="28"/>
+      <c r="J60" s="28"/>
+      <c r="K60" s="29"/>
     </row>
     <row r="61">
       <c r="B61" s="1" t="s">
@@ -8520,11 +8523,11 @@
       <c r="E61" s="1">
         <v>0.916437840058194</v>
       </c>
-      <c r="J61" s="27"/>
-      <c r="K61" s="28"/>
+      <c r="J61" s="28"/>
+      <c r="K61" s="29"/>
     </row>
     <row r="62">
-      <c r="A62" s="25"/>
+      <c r="A62" s="26"/>
       <c r="B62" s="1" t="s">
         <v>17</v>
       </c>
@@ -8537,11 +8540,11 @@
       <c r="E62" s="1">
         <v>0.699786398186203</v>
       </c>
-      <c r="J62" s="27"/>
-      <c r="K62" s="28"/>
+      <c r="J62" s="28"/>
+      <c r="K62" s="29"/>
     </row>
     <row r="63">
-      <c r="A63" s="26" t="s">
+      <c r="A63" s="27" t="s">
         <v>338</v>
       </c>
       <c r="C63" s="1" t="s">
@@ -8566,8 +8569,8 @@
       <c r="E64" s="1">
         <v>0.6918024201</v>
       </c>
-      <c r="J64" s="27"/>
-      <c r="K64" s="28"/>
+      <c r="J64" s="28"/>
+      <c r="K64" s="29"/>
     </row>
     <row r="65">
       <c r="B65" s="1" t="s">
@@ -8582,8 +8585,8 @@
       <c r="E65" s="1">
         <v>0.9907632305</v>
       </c>
-      <c r="J65" s="27"/>
-      <c r="K65" s="28"/>
+      <c r="J65" s="28"/>
+      <c r="K65" s="29"/>
     </row>
     <row r="66">
       <c r="B66" s="1" t="s">
@@ -8598,8 +8601,8 @@
       <c r="E66" s="1">
         <v>0.82483737</v>
       </c>
-      <c r="J66" s="27"/>
-      <c r="K66" s="28"/>
+      <c r="J66" s="28"/>
+      <c r="K66" s="29"/>
     </row>
     <row r="67">
       <c r="A67" s="1" t="s">
@@ -8617,8 +8620,8 @@
       <c r="E67" s="1">
         <v>0.6935956635</v>
       </c>
-      <c r="J67" s="27"/>
-      <c r="K67" s="28"/>
+      <c r="J67" s="28"/>
+      <c r="K67" s="29"/>
     </row>
     <row r="68">
       <c r="B68" s="1" t="s">
@@ -8633,8 +8636,8 @@
       <c r="E68" s="1">
         <v>1.0573650168</v>
       </c>
-      <c r="J68" s="27"/>
-      <c r="K68" s="28"/>
+      <c r="J68" s="28"/>
+      <c r="K68" s="29"/>
     </row>
     <row r="69">
       <c r="B69" s="1" t="s">
@@ -8649,8 +8652,8 @@
       <c r="E69" s="1">
         <v>0.9511330905</v>
       </c>
-      <c r="J69" s="27"/>
-      <c r="K69" s="28"/>
+      <c r="J69" s="28"/>
+      <c r="K69" s="29"/>
     </row>
     <row r="70">
       <c r="A70" s="1" t="s">
@@ -8668,8 +8671,8 @@
       <c r="E70" s="1">
         <v>0.6652188953</v>
       </c>
-      <c r="J70" s="27"/>
-      <c r="K70" s="28"/>
+      <c r="J70" s="28"/>
+      <c r="K70" s="29"/>
     </row>
     <row r="71">
       <c r="B71" s="1" t="s">
@@ -8684,8 +8687,8 @@
       <c r="E71" s="1">
         <v>0.9292311212</v>
       </c>
-      <c r="J71" s="27"/>
-      <c r="K71" s="28"/>
+      <c r="J71" s="28"/>
+      <c r="K71" s="29"/>
     </row>
     <row r="72">
       <c r="B72" s="1" t="s">
@@ -8700,8 +8703,8 @@
       <c r="E72" s="1">
         <v>0.9478648152</v>
       </c>
-      <c r="J72" s="27"/>
-      <c r="K72" s="28"/>
+      <c r="J72" s="28"/>
+      <c r="K72" s="29"/>
     </row>
     <row r="73">
       <c r="A73" s="1" t="s">
@@ -8719,8 +8722,8 @@
       <c r="E73" s="1">
         <v>0.6785552684</v>
       </c>
-      <c r="J73" s="27"/>
-      <c r="K73" s="28"/>
+      <c r="J73" s="28"/>
+      <c r="K73" s="29"/>
     </row>
     <row r="74">
       <c r="B74" s="1" t="s">
@@ -8735,8 +8738,8 @@
       <c r="E74" s="1">
         <v>0.8446965494</v>
       </c>
-      <c r="J74" s="27"/>
-      <c r="K74" s="28"/>
+      <c r="J74" s="28"/>
+      <c r="K74" s="29"/>
     </row>
     <row r="75">
       <c r="B75" s="1" t="s">
@@ -8751,8 +8754,8 @@
       <c r="E75" s="1">
         <v>0.7181710076</v>
       </c>
-      <c r="J75" s="27"/>
-      <c r="K75" s="28"/>
+      <c r="J75" s="28"/>
+      <c r="K75" s="29"/>
     </row>
     <row r="76">
       <c r="A76" s="1" t="s">
@@ -8770,8 +8773,8 @@
       <c r="E76" s="1">
         <v>0.7404798108</v>
       </c>
-      <c r="J76" s="27"/>
-      <c r="K76" s="28"/>
+      <c r="J76" s="28"/>
+      <c r="K76" s="29"/>
     </row>
     <row r="77">
       <c r="B77" s="1" t="s">
@@ -8786,8 +8789,8 @@
       <c r="E77" s="1">
         <v>1.0419580617</v>
       </c>
-      <c r="J77" s="27"/>
-      <c r="K77" s="28"/>
+      <c r="J77" s="28"/>
+      <c r="K77" s="29"/>
     </row>
     <row r="78">
       <c r="B78" s="1" t="s">
@@ -8802,8 +8805,8 @@
       <c r="E78" s="1">
         <v>0.6789101833</v>
       </c>
-      <c r="J78" s="27"/>
-      <c r="K78" s="28"/>
+      <c r="J78" s="28"/>
+      <c r="K78" s="29"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="s">
@@ -8821,8 +8824,8 @@
       <c r="E79" s="1">
         <v>0.722388690672348</v>
       </c>
-      <c r="J79" s="27"/>
-      <c r="K79" s="28"/>
+      <c r="J79" s="28"/>
+      <c r="K79" s="29"/>
     </row>
     <row r="80">
       <c r="B80" s="1" t="s">
@@ -8837,8 +8840,8 @@
       <c r="E80" s="1">
         <v>0.875038589623464</v>
       </c>
-      <c r="J80" s="27"/>
-      <c r="K80" s="28"/>
+      <c r="J80" s="28"/>
+      <c r="K80" s="29"/>
     </row>
     <row r="81">
       <c r="B81" s="1" t="s">
@@ -8853,8 +8856,8 @@
       <c r="E81" s="1">
         <v>1.39046467117004</v>
       </c>
-      <c r="J81" s="27"/>
-      <c r="K81" s="28"/>
+      <c r="J81" s="28"/>
+      <c r="K81" s="29"/>
     </row>
     <row r="82">
       <c r="A82" s="1" t="s">
@@ -8872,8 +8875,8 @@
       <c r="E82" s="1">
         <v>0.6938557598</v>
       </c>
-      <c r="J82" s="27"/>
-      <c r="K82" s="28"/>
+      <c r="J82" s="28"/>
+      <c r="K82" s="29"/>
     </row>
     <row r="83">
       <c r="B83" s="1" t="s">
@@ -8888,8 +8891,8 @@
       <c r="E83" s="1">
         <v>0.8980291949</v>
       </c>
-      <c r="J83" s="27"/>
-      <c r="K83" s="28"/>
+      <c r="J83" s="28"/>
+      <c r="K83" s="29"/>
     </row>
     <row r="84">
       <c r="B84" s="1" t="s">
@@ -8904,8 +8907,8 @@
       <c r="E84" s="1">
         <v>0.7200478942</v>
       </c>
-      <c r="J84" s="27"/>
-      <c r="K84" s="28"/>
+      <c r="J84" s="28"/>
+      <c r="K84" s="29"/>
     </row>
     <row r="85">
       <c r="A85" s="1" t="s">
@@ -8923,8 +8926,8 @@
       <c r="E85" s="1">
         <v>0.6759991876</v>
       </c>
-      <c r="J85" s="27"/>
-      <c r="K85" s="28"/>
+      <c r="J85" s="28"/>
+      <c r="K85" s="29"/>
     </row>
     <row r="86">
       <c r="B86" s="1" t="s">
@@ -8939,8 +8942,8 @@
       <c r="E86" s="1">
         <v>1.0596259539</v>
       </c>
-      <c r="J86" s="27"/>
-      <c r="K86" s="28"/>
+      <c r="J86" s="28"/>
+      <c r="K86" s="29"/>
     </row>
     <row r="87">
       <c r="B87" s="1" t="s">
@@ -8955,8 +8958,8 @@
       <c r="E87" s="1">
         <v>0.7635727213</v>
       </c>
-      <c r="J87" s="27"/>
-      <c r="K87" s="28"/>
+      <c r="J87" s="28"/>
+      <c r="K87" s="29"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="s">
@@ -8974,8 +8977,8 @@
       <c r="E88" s="1">
         <v>0.617555902263986</v>
       </c>
-      <c r="J88" s="27"/>
-      <c r="K88" s="28"/>
+      <c r="J88" s="28"/>
+      <c r="K88" s="29"/>
     </row>
     <row r="89">
       <c r="B89" s="1" t="s">
@@ -8990,8 +8993,8 @@
       <c r="E89" s="1">
         <v>1.05526514702039</v>
       </c>
-      <c r="J89" s="27"/>
-      <c r="K89" s="28"/>
+      <c r="J89" s="28"/>
+      <c r="K89" s="29"/>
     </row>
     <row r="90">
       <c r="B90" s="1" t="s">
@@ -9006,8 +9009,8 @@
       <c r="E90" s="1">
         <v>0.7068303251794</v>
       </c>
-      <c r="J90" s="27"/>
-      <c r="K90" s="28"/>
+      <c r="J90" s="28"/>
+      <c r="K90" s="29"/>
     </row>
     <row r="91">
       <c r="A91" s="1" t="s">
@@ -9025,8 +9028,8 @@
       <c r="E91" s="1">
         <v>0.648114875180265</v>
       </c>
-      <c r="J91" s="27"/>
-      <c r="K91" s="28"/>
+      <c r="J91" s="28"/>
+      <c r="K91" s="29"/>
     </row>
     <row r="92">
       <c r="B92" s="1" t="s">
@@ -9041,8 +9044,8 @@
       <c r="E92" s="1">
         <v>0.898316619561315</v>
       </c>
-      <c r="J92" s="27"/>
-      <c r="K92" s="28"/>
+      <c r="J92" s="28"/>
+      <c r="K92" s="29"/>
     </row>
     <row r="93">
       <c r="B93" s="1" t="s">
@@ -9057,8 +9060,8 @@
       <c r="E93" s="1">
         <v>0.729357808900581</v>
       </c>
-      <c r="J93" s="27"/>
-      <c r="K93" s="28"/>
+      <c r="J93" s="28"/>
+      <c r="K93" s="29"/>
     </row>
     <row r="94">
       <c r="A94" s="1" t="s">
@@ -9076,8 +9079,8 @@
       <c r="E94" s="1">
         <v>0.6756369776</v>
       </c>
-      <c r="J94" s="27"/>
-      <c r="K94" s="28"/>
+      <c r="J94" s="28"/>
+      <c r="K94" s="29"/>
     </row>
     <row r="95">
       <c r="B95" s="1" t="s">
@@ -9092,8 +9095,8 @@
       <c r="E95" s="1">
         <v>1.0959080646</v>
       </c>
-      <c r="J95" s="27"/>
-      <c r="K95" s="28"/>
+      <c r="J95" s="28"/>
+      <c r="K95" s="29"/>
     </row>
     <row r="96">
       <c r="B96" s="1" t="s">
@@ -9108,10 +9111,10 @@
       <c r="E96" s="1">
         <v>0.774511134</v>
       </c>
-      <c r="J96" s="27"/>
-      <c r="K96" s="28"/>
-      <c r="N96" s="33"/>
-      <c r="O96" s="33"/>
+      <c r="J96" s="28"/>
+      <c r="K96" s="29"/>
+      <c r="N96" s="34"/>
+      <c r="O96" s="34"/>
     </row>
     <row r="97">
       <c r="A97" s="1" t="s">
@@ -9120,7 +9123,7 @@
       <c r="B97" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C97" s="22">
+      <c r="C97" s="23">
         <v>4.0</v>
       </c>
       <c r="D97" s="1">
@@ -9129,10 +9132,10 @@
       <c r="E97" s="1">
         <v>0.7324887419</v>
       </c>
-      <c r="J97" s="27"/>
-      <c r="K97" s="28"/>
-      <c r="N97" s="33"/>
-      <c r="O97" s="33"/>
+      <c r="J97" s="28"/>
+      <c r="K97" s="29"/>
+      <c r="N97" s="34"/>
+      <c r="O97" s="34"/>
     </row>
     <row r="98">
       <c r="B98" s="1" t="s">
@@ -9147,10 +9150,10 @@
       <c r="E98" s="1">
         <v>1.0326041155</v>
       </c>
-      <c r="J98" s="27"/>
-      <c r="K98" s="28"/>
-      <c r="N98" s="33"/>
-      <c r="O98" s="33"/>
+      <c r="J98" s="28"/>
+      <c r="K98" s="29"/>
+      <c r="N98" s="34"/>
+      <c r="O98" s="34"/>
     </row>
     <row r="99">
       <c r="B99" s="1" t="s">
@@ -9165,10 +9168,10 @@
       <c r="E99" s="1">
         <v>0.7585566574</v>
       </c>
-      <c r="J99" s="27"/>
-      <c r="K99" s="28"/>
-      <c r="N99" s="33"/>
-      <c r="O99" s="33"/>
+      <c r="J99" s="28"/>
+      <c r="K99" s="29"/>
+      <c r="N99" s="34"/>
+      <c r="O99" s="34"/>
     </row>
     <row r="100">
       <c r="A100" s="1" t="s">
@@ -9177,7 +9180,7 @@
       <c r="B100" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C100" s="22">
+      <c r="C100" s="23">
         <v>2.0</v>
       </c>
       <c r="D100" s="1">
@@ -9186,10 +9189,10 @@
       <c r="E100" s="1">
         <v>0.6739674954</v>
       </c>
-      <c r="J100" s="27"/>
-      <c r="K100" s="28"/>
-      <c r="N100" s="33"/>
-      <c r="O100" s="33"/>
+      <c r="J100" s="28"/>
+      <c r="K100" s="29"/>
+      <c r="N100" s="34"/>
+      <c r="O100" s="34"/>
     </row>
     <row r="101">
       <c r="B101" s="1" t="s">
@@ -9204,10 +9207,10 @@
       <c r="E101" s="1">
         <v>0.9697900619</v>
       </c>
-      <c r="J101" s="27"/>
-      <c r="K101" s="28"/>
-      <c r="N101" s="33"/>
-      <c r="O101" s="33"/>
+      <c r="J101" s="28"/>
+      <c r="K101" s="29"/>
+      <c r="N101" s="34"/>
+      <c r="O101" s="34"/>
     </row>
     <row r="102">
       <c r="B102" s="1" t="s">
@@ -9222,10 +9225,10 @@
       <c r="E102" s="1">
         <v>1.1288435358</v>
       </c>
-      <c r="J102" s="27"/>
-      <c r="K102" s="28"/>
-      <c r="N102" s="33"/>
-      <c r="O102" s="33"/>
+      <c r="J102" s="28"/>
+      <c r="K102" s="29"/>
+      <c r="N102" s="34"/>
+      <c r="O102" s="34"/>
     </row>
     <row r="103">
       <c r="A103" s="1" t="s">
@@ -9234,7 +9237,7 @@
       <c r="B103" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C103" s="22">
+      <c r="C103" s="23">
         <v>3.0</v>
       </c>
       <c r="D103" s="1">
@@ -9243,10 +9246,10 @@
       <c r="E103" s="1">
         <v>0.6695189558</v>
       </c>
-      <c r="J103" s="27"/>
-      <c r="K103" s="28"/>
-      <c r="N103" s="33"/>
-      <c r="O103" s="33"/>
+      <c r="J103" s="28"/>
+      <c r="K103" s="29"/>
+      <c r="N103" s="34"/>
+      <c r="O103" s="34"/>
     </row>
     <row r="104">
       <c r="B104" s="1" t="s">
@@ -9261,10 +9264,10 @@
       <c r="E104" s="1">
         <v>0.8664588519</v>
       </c>
-      <c r="J104" s="27"/>
-      <c r="K104" s="28"/>
-      <c r="N104" s="33"/>
-      <c r="O104" s="33"/>
+      <c r="J104" s="28"/>
+      <c r="K104" s="29"/>
+      <c r="N104" s="34"/>
+      <c r="O104" s="34"/>
     </row>
     <row r="105">
       <c r="B105" s="1" t="s">
@@ -9273,16 +9276,16 @@
       <c r="C105" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="D105" s="22">
+      <c r="D105" s="23">
         <v>1.77076115752053E9</v>
       </c>
-      <c r="E105" s="22">
+      <c r="E105" s="23">
         <v>1.0378559732</v>
       </c>
-      <c r="J105" s="27"/>
-      <c r="K105" s="28"/>
-      <c r="N105" s="33"/>
-      <c r="O105" s="33"/>
+      <c r="J105" s="28"/>
+      <c r="K105" s="29"/>
+      <c r="N105" s="34"/>
+      <c r="O105" s="34"/>
     </row>
     <row r="106">
       <c r="A106" s="1" t="s">
@@ -9291,7 +9294,7 @@
       <c r="B106" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C106" s="22">
+      <c r="C106" s="23">
         <v>5.0</v>
       </c>
       <c r="D106" s="1">
@@ -9300,10 +9303,10 @@
       <c r="E106" s="1">
         <v>0.7058638883</v>
       </c>
-      <c r="J106" s="27"/>
-      <c r="K106" s="28"/>
-      <c r="N106" s="33"/>
-      <c r="O106" s="33"/>
+      <c r="J106" s="28"/>
+      <c r="K106" s="29"/>
+      <c r="N106" s="34"/>
+      <c r="O106" s="34"/>
     </row>
     <row r="107">
       <c r="B107" s="1" t="s">
@@ -9318,10 +9321,10 @@
       <c r="E107" s="1">
         <v>1.0436391403</v>
       </c>
-      <c r="J107" s="27"/>
-      <c r="K107" s="28"/>
-      <c r="N107" s="33"/>
-      <c r="O107" s="33"/>
+      <c r="J107" s="28"/>
+      <c r="K107" s="29"/>
+      <c r="N107" s="34"/>
+      <c r="O107" s="34"/>
     </row>
     <row r="108">
       <c r="B108" s="1" t="s">
@@ -9336,10 +9339,10 @@
       <c r="E108" s="1">
         <v>0.7070192763</v>
       </c>
-      <c r="J108" s="27"/>
-      <c r="K108" s="28"/>
-      <c r="N108" s="33"/>
-      <c r="O108" s="33"/>
+      <c r="J108" s="28"/>
+      <c r="K108" s="29"/>
+      <c r="N108" s="34"/>
+      <c r="O108" s="34"/>
     </row>
     <row r="109">
       <c r="A109" s="1" t="s">
@@ -9357,8 +9360,8 @@
       <c r="E109" s="1">
         <v>0.6993529493</v>
       </c>
-      <c r="J109" s="27"/>
-      <c r="K109" s="28"/>
+      <c r="J109" s="28"/>
+      <c r="K109" s="29"/>
     </row>
     <row r="110">
       <c r="B110" s="1" t="s">
@@ -9373,8 +9376,8 @@
       <c r="E110" s="1">
         <v>0.8183505199</v>
       </c>
-      <c r="J110" s="27"/>
-      <c r="K110" s="28"/>
+      <c r="J110" s="28"/>
+      <c r="K110" s="29"/>
     </row>
     <row r="111">
       <c r="B111" s="1" t="s">
@@ -9389,18 +9392,18 @@
       <c r="E111" s="1">
         <v>0.7157412862</v>
       </c>
-      <c r="J111" s="27"/>
-      <c r="K111" s="28"/>
+      <c r="J111" s="28"/>
+      <c r="K111" s="29"/>
     </row>
     <row r="112">
-      <c r="A112" s="26" t="s">
+      <c r="A112" s="27" t="s">
         <v>339</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="J112" s="27"/>
-      <c r="K112" s="28"/>
+      <c r="J112" s="28"/>
+      <c r="K112" s="29"/>
     </row>
     <row r="113">
       <c r="A113" s="1" t="s">
@@ -9418,7 +9421,7 @@
       <c r="E113" s="1">
         <v>0.7631135756</v>
       </c>
-      <c r="J113" s="27"/>
+      <c r="J113" s="28"/>
     </row>
     <row r="114">
       <c r="B114" s="1" t="s">
@@ -9433,7 +9436,7 @@
       <c r="E114" s="1">
         <v>0.7938452464</v>
       </c>
-      <c r="J114" s="27"/>
+      <c r="J114" s="28"/>
     </row>
     <row r="115">
       <c r="A115" s="1" t="s">
@@ -9451,7 +9454,7 @@
       <c r="E115" s="1">
         <v>0.7634124267</v>
       </c>
-      <c r="J115" s="27"/>
+      <c r="J115" s="28"/>
     </row>
     <row r="116">
       <c r="B116" s="1" t="s">
@@ -9466,7 +9469,7 @@
       <c r="E116" s="1">
         <v>0.8280248969</v>
       </c>
-      <c r="J116" s="27"/>
+      <c r="J116" s="28"/>
     </row>
     <row r="117">
       <c r="A117" s="1" t="s">
@@ -9487,7 +9490,7 @@
       <c r="F117" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="J117" s="27"/>
+      <c r="J117" s="28"/>
     </row>
     <row r="118">
       <c r="B118" s="1" t="s">
@@ -9502,7 +9505,7 @@
       <c r="E118" s="1">
         <v>1.1734408999</v>
       </c>
-      <c r="J118" s="27"/>
+      <c r="J118" s="28"/>
     </row>
     <row r="119">
       <c r="A119" s="1" t="s">
@@ -9520,7 +9523,7 @@
       <c r="E119" s="1">
         <v>0.7402349295</v>
       </c>
-      <c r="J119" s="27"/>
+      <c r="J119" s="28"/>
     </row>
     <row r="120">
       <c r="B120" s="1" t="s">
@@ -9535,7 +9538,7 @@
       <c r="E120" s="1">
         <v>1.2271572646</v>
       </c>
-      <c r="J120" s="27"/>
+      <c r="J120" s="28"/>
     </row>
     <row r="121">
       <c r="A121" s="1" t="s">
@@ -9553,7 +9556,7 @@
       <c r="E121" s="1">
         <v>0.760669434604679</v>
       </c>
-      <c r="J121" s="27"/>
+      <c r="J121" s="28"/>
     </row>
     <row r="122">
       <c r="B122" s="1" t="s">
@@ -9568,7 +9571,7 @@
       <c r="E122" s="1">
         <v>1.09487519747564</v>
       </c>
-      <c r="J122" s="27"/>
+      <c r="J122" s="28"/>
     </row>
     <row r="123">
       <c r="A123" s="1" t="s">
@@ -9589,7 +9592,7 @@
       <c r="F123" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="J123" s="27"/>
+      <c r="J123" s="28"/>
     </row>
     <row r="124">
       <c r="B124" s="1" t="s">
@@ -9604,7 +9607,7 @@
       <c r="E124" s="1">
         <v>1.0746031465</v>
       </c>
-      <c r="J124" s="27"/>
+      <c r="J124" s="28"/>
     </row>
     <row r="125">
       <c r="A125" s="1" t="s">
@@ -9622,7 +9625,7 @@
       <c r="E125" s="1">
         <v>0.767427665351752</v>
       </c>
-      <c r="J125" s="27"/>
+      <c r="J125" s="28"/>
     </row>
     <row r="126">
       <c r="B126" s="1" t="s">
@@ -9637,7 +9640,7 @@
       <c r="E126" s="1">
         <v>1.14565358823941</v>
       </c>
-      <c r="J126" s="27"/>
+      <c r="J126" s="28"/>
     </row>
     <row r="127">
       <c r="A127" s="1" t="s">
@@ -9655,7 +9658,7 @@
       <c r="E127" s="1">
         <v>0.8090669306</v>
       </c>
-      <c r="J127" s="27"/>
+      <c r="J127" s="28"/>
     </row>
     <row r="128">
       <c r="B128" s="1" t="s">
@@ -9670,7 +9673,7 @@
       <c r="E128" s="1">
         <v>0.9732260447</v>
       </c>
-      <c r="J128" s="27"/>
+      <c r="J128" s="28"/>
     </row>
     <row r="129">
       <c r="A129" s="1" t="s">
@@ -9688,7 +9691,7 @@
       <c r="E129" s="1">
         <v>0.834754076</v>
       </c>
-      <c r="J129" s="27"/>
+      <c r="J129" s="28"/>
     </row>
     <row r="130">
       <c r="B130" s="1" t="s">
@@ -9703,7 +9706,7 @@
       <c r="E130" s="1">
         <v>0.9683953042</v>
       </c>
-      <c r="J130" s="27"/>
+      <c r="J130" s="28"/>
     </row>
     <row r="131">
       <c r="A131" s="1" t="s">
@@ -9721,7 +9724,7 @@
       <c r="E131" s="1">
         <v>0.7852399325</v>
       </c>
-      <c r="J131" s="27"/>
+      <c r="J131" s="28"/>
     </row>
     <row r="132">
       <c r="B132" s="1" t="s">
@@ -9736,7 +9739,7 @@
       <c r="E132" s="1">
         <v>0.956274921</v>
       </c>
-      <c r="J132" s="27"/>
+      <c r="J132" s="28"/>
     </row>
     <row r="133">
       <c r="A133" s="1" t="s">
@@ -9754,7 +9757,7 @@
       <c r="E133" s="1">
         <v>0.778745713440709</v>
       </c>
-      <c r="J133" s="27"/>
+      <c r="J133" s="28"/>
     </row>
     <row r="134">
       <c r="B134" s="1" t="s">
@@ -9769,7 +9772,7 @@
       <c r="E134" s="1">
         <v>1.08833633722298</v>
       </c>
-      <c r="J134" s="27"/>
+      <c r="J134" s="28"/>
     </row>
     <row r="135">
       <c r="A135" s="1" t="s">
@@ -9787,7 +9790,7 @@
       <c r="E135" s="1">
         <v>0.7791491994</v>
       </c>
-      <c r="J135" s="27"/>
+      <c r="J135" s="28"/>
     </row>
     <row r="136">
       <c r="B136" s="1" t="s">
@@ -9802,7 +9805,7 @@
       <c r="E136" s="1">
         <v>1.0405958084</v>
       </c>
-      <c r="J136" s="27"/>
+      <c r="J136" s="28"/>
     </row>
     <row r="137">
       <c r="A137" s="1" t="s">
@@ -9820,7 +9823,7 @@
       <c r="E137" s="1">
         <v>0.728108161</v>
       </c>
-      <c r="J137" s="27"/>
+      <c r="J137" s="28"/>
     </row>
     <row r="138">
       <c r="B138" s="1" t="s">
@@ -9835,7 +9838,7 @@
       <c r="E138" s="1">
         <v>1.1061910473</v>
       </c>
-      <c r="J138" s="27"/>
+      <c r="J138" s="28"/>
     </row>
     <row r="139">
       <c r="A139" s="1" t="s">
@@ -9853,7 +9856,7 @@
       <c r="E139" s="1">
         <v>0.7360634351</v>
       </c>
-      <c r="J139" s="27"/>
+      <c r="J139" s="28"/>
     </row>
     <row r="140">
       <c r="B140" s="1" t="s">
@@ -9868,7 +9871,7 @@
       <c r="E140" s="1">
         <v>0.9018015842</v>
       </c>
-      <c r="J140" s="27"/>
+      <c r="J140" s="28"/>
     </row>
     <row r="141">
       <c r="A141" s="1" t="s">
@@ -9886,7 +9889,7 @@
       <c r="E141" s="1">
         <v>0.7616601807</v>
       </c>
-      <c r="J141" s="27"/>
+      <c r="J141" s="28"/>
     </row>
     <row r="142">
       <c r="B142" s="1" t="s">
@@ -9901,7 +9904,7 @@
       <c r="E142" s="1">
         <v>1.110426904</v>
       </c>
-      <c r="J142" s="27"/>
+      <c r="J142" s="28"/>
     </row>
     <row r="143">
       <c r="A143" s="1" t="s">
@@ -9919,7 +9922,7 @@
       <c r="E143" s="1">
         <v>0.746394721629512</v>
       </c>
-      <c r="J143" s="27"/>
+      <c r="J143" s="28"/>
     </row>
     <row r="144">
       <c r="B144" s="1" t="s">
@@ -9934,7 +9937,7 @@
       <c r="E144" s="1">
         <v>1.0645070887192</v>
       </c>
-      <c r="J144" s="27"/>
+      <c r="J144" s="28"/>
     </row>
     <row r="145">
       <c r="A145" s="1" t="s">
@@ -9955,7 +9958,7 @@
       <c r="F145" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="J145" s="27"/>
+      <c r="J145" s="28"/>
     </row>
     <row r="146">
       <c r="B146" s="1" t="s">
@@ -9970,7 +9973,7 @@
       <c r="E146" s="1">
         <v>1.8035336372</v>
       </c>
-      <c r="J146" s="27"/>
+      <c r="J146" s="28"/>
     </row>
     <row r="147">
       <c r="A147" s="1" t="s">
@@ -9988,7 +9991,7 @@
       <c r="E147" s="1">
         <v>0.7706837071</v>
       </c>
-      <c r="J147" s="27"/>
+      <c r="J147" s="28"/>
     </row>
     <row r="148">
       <c r="B148" s="1" t="s">
@@ -10003,7 +10006,7 @@
       <c r="E148" s="1">
         <v>1.4951655779</v>
       </c>
-      <c r="J148" s="27"/>
+      <c r="J148" s="28"/>
     </row>
     <row r="149">
       <c r="A149" s="1" t="s">
@@ -10021,7 +10024,7 @@
       <c r="E149" s="1">
         <v>0.7332467526</v>
       </c>
-      <c r="J149" s="27"/>
+      <c r="J149" s="28"/>
     </row>
     <row r="150">
       <c r="B150" s="1" t="s">
@@ -10036,7 +10039,7 @@
       <c r="E150" s="1">
         <v>1.1810047602</v>
       </c>
-      <c r="J150" s="27"/>
+      <c r="J150" s="28"/>
     </row>
     <row r="151">
       <c r="A151" s="1" t="s">
@@ -10054,7 +10057,7 @@
       <c r="E151" s="1">
         <v>0.731822272290115</v>
       </c>
-      <c r="J151" s="27"/>
+      <c r="J151" s="28"/>
     </row>
     <row r="152">
       <c r="B152" s="1" t="s">
@@ -10069,31 +10072,31 @@
       <c r="E152" s="1">
         <v>0.85893421798748</v>
       </c>
-      <c r="J152" s="27"/>
+      <c r="J152" s="28"/>
     </row>
     <row r="153">
-      <c r="J153" s="27"/>
+      <c r="J153" s="28"/>
     </row>
     <row r="154">
-      <c r="J154" s="27"/>
+      <c r="J154" s="28"/>
     </row>
     <row r="155">
-      <c r="J155" s="27"/>
+      <c r="J155" s="28"/>
     </row>
     <row r="156">
-      <c r="J156" s="27"/>
+      <c r="J156" s="28"/>
     </row>
     <row r="157">
-      <c r="J157" s="27"/>
+      <c r="J157" s="28"/>
     </row>
     <row r="158">
-      <c r="J158" s="27"/>
+      <c r="J158" s="28"/>
     </row>
     <row r="159">
-      <c r="J159" s="27"/>
+      <c r="J159" s="28"/>
     </row>
     <row r="160">
-      <c r="J160" s="27"/>
+      <c r="J160" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>